<commit_message>
Update rasters en R scripts
</commit_message>
<xml_diff>
--- a/data/input/Excel_files/Soortenlijst_Maatwerkgebieden_Gefilterd.xlsx
+++ b/data/input/Excel_files/Soortenlijst_Maatwerkgebieden_Gefilterd.xlsx
@@ -5,7 +5,7 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bert_vanhecke\PycharmProjects\PythonProject\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bert_vanhecke\Documents\Soortenbehoud\arpl\data\input\Excel_files\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -1507,16 +1507,16 @@
         <v>172</v>
       </c>
       <c r="B11" t="s">
-        <v>185</v>
+        <v>173</v>
       </c>
       <c r="C11" t="s">
-        <v>186</v>
+        <v>174</v>
       </c>
       <c r="D11" t="s">
         <v>14</v>
       </c>
       <c r="E11" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F11">
         <v>0</v>
@@ -1525,10 +1525,10 @@
         <v>0</v>
       </c>
       <c r="H11">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I11">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J11">
         <v>1</v>
@@ -2137,10 +2137,10 @@
         <v>172</v>
       </c>
       <c r="B29" t="s">
-        <v>187</v>
+        <v>175</v>
       </c>
       <c r="C29" t="s">
-        <v>188</v>
+        <v>176</v>
       </c>
       <c r="D29" t="s">
         <v>14</v>
@@ -2149,22 +2149,22 @@
         <v>15</v>
       </c>
       <c r="F29">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G29">
         <v>0</v>
       </c>
       <c r="H29">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I29">
         <v>1</v>
       </c>
       <c r="J29">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K29">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="30" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
@@ -3257,10 +3257,10 @@
         <v>172</v>
       </c>
       <c r="B61" t="s">
-        <v>205</v>
+        <v>177</v>
       </c>
       <c r="C61" t="s">
-        <v>206</v>
+        <v>178</v>
       </c>
       <c r="D61" t="s">
         <v>14</v>
@@ -3272,7 +3272,7 @@
         <v>0</v>
       </c>
       <c r="G61">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H61">
         <v>0</v>
@@ -3284,7 +3284,7 @@
         <v>1</v>
       </c>
       <c r="K61">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="62" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
@@ -3817,16 +3817,16 @@
         <v>172</v>
       </c>
       <c r="B77" t="s">
-        <v>173</v>
+        <v>179</v>
       </c>
       <c r="C77" t="s">
-        <v>174</v>
+        <v>180</v>
       </c>
       <c r="D77" t="s">
         <v>14</v>
       </c>
       <c r="E77" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F77">
         <v>0</v>
@@ -3835,10 +3835,10 @@
         <v>0</v>
       </c>
       <c r="H77">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I77">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J77">
         <v>1</v>
@@ -3852,10 +3852,10 @@
         <v>172</v>
       </c>
       <c r="B78" t="s">
-        <v>175</v>
+        <v>181</v>
       </c>
       <c r="C78" t="s">
-        <v>176</v>
+        <v>182</v>
       </c>
       <c r="D78" t="s">
         <v>14</v>
@@ -3864,16 +3864,16 @@
         <v>15</v>
       </c>
       <c r="F78">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G78">
         <v>0</v>
       </c>
       <c r="H78">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I78">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J78">
         <v>1</v>
@@ -3887,10 +3887,10 @@
         <v>172</v>
       </c>
       <c r="B79" t="s">
-        <v>177</v>
+        <v>183</v>
       </c>
       <c r="C79" t="s">
-        <v>178</v>
+        <v>184</v>
       </c>
       <c r="D79" t="s">
         <v>14</v>
@@ -3899,16 +3899,16 @@
         <v>15</v>
       </c>
       <c r="F79">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G79">
         <v>0</v>
       </c>
       <c r="H79">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I79">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J79">
         <v>1</v>
@@ -3922,10 +3922,10 @@
         <v>172</v>
       </c>
       <c r="B80" t="s">
-        <v>179</v>
+        <v>185</v>
       </c>
       <c r="C80" t="s">
-        <v>180</v>
+        <v>186</v>
       </c>
       <c r="D80" t="s">
         <v>14</v>
@@ -3952,15 +3952,15 @@
         <v>0</v>
       </c>
     </row>
-    <row r="81" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
         <v>172</v>
       </c>
       <c r="B81" t="s">
-        <v>181</v>
+        <v>187</v>
       </c>
       <c r="C81" t="s">
-        <v>182</v>
+        <v>188</v>
       </c>
       <c r="D81" t="s">
         <v>14</v>
@@ -3978,13 +3978,13 @@
         <v>0</v>
       </c>
       <c r="I81">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J81">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K81">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="82" spans="1:11" x14ac:dyDescent="0.3">
@@ -3992,10 +3992,10 @@
         <v>172</v>
       </c>
       <c r="B82" t="s">
-        <v>183</v>
+        <v>189</v>
       </c>
       <c r="C82" t="s">
-        <v>184</v>
+        <v>190</v>
       </c>
       <c r="D82" t="s">
         <v>14</v>
@@ -4010,7 +4010,7 @@
         <v>0</v>
       </c>
       <c r="H82">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I82">
         <v>0</v>
@@ -4062,34 +4062,34 @@
         <v>172</v>
       </c>
       <c r="B84" t="s">
-        <v>211</v>
+        <v>191</v>
       </c>
       <c r="C84" t="s">
-        <v>212</v>
+        <v>192</v>
       </c>
       <c r="D84" t="s">
         <v>14</v>
       </c>
       <c r="E84" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F84">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G84">
         <v>1</v>
       </c>
       <c r="H84">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I84">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J84">
         <v>1</v>
       </c>
       <c r="K84">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="85" spans="1:11" x14ac:dyDescent="0.3">
@@ -4097,10 +4097,10 @@
         <v>172</v>
       </c>
       <c r="B85" t="s">
-        <v>189</v>
+        <v>193</v>
       </c>
       <c r="C85" t="s">
-        <v>190</v>
+        <v>194</v>
       </c>
       <c r="D85" t="s">
         <v>14</v>
@@ -4132,10 +4132,10 @@
         <v>172</v>
       </c>
       <c r="B86" t="s">
-        <v>191</v>
+        <v>195</v>
       </c>
       <c r="C86" t="s">
-        <v>192</v>
+        <v>196</v>
       </c>
       <c r="D86" t="s">
         <v>14</v>
@@ -4147,10 +4147,10 @@
         <v>0</v>
       </c>
       <c r="G86">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H86">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I86">
         <v>0</v>
@@ -4167,19 +4167,19 @@
         <v>172</v>
       </c>
       <c r="B87" t="s">
-        <v>193</v>
+        <v>197</v>
       </c>
       <c r="C87" t="s">
-        <v>194</v>
+        <v>198</v>
       </c>
       <c r="D87" t="s">
         <v>14</v>
       </c>
       <c r="E87" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F87">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G87">
         <v>0</v>
@@ -4202,10 +4202,10 @@
         <v>172</v>
       </c>
       <c r="B88" t="s">
-        <v>195</v>
+        <v>199</v>
       </c>
       <c r="C88" t="s">
-        <v>196</v>
+        <v>200</v>
       </c>
       <c r="D88" t="s">
         <v>14</v>
@@ -4214,7 +4214,7 @@
         <v>15</v>
       </c>
       <c r="F88">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G88">
         <v>0</v>
@@ -4237,16 +4237,16 @@
         <v>172</v>
       </c>
       <c r="B89" t="s">
-        <v>197</v>
+        <v>201</v>
       </c>
       <c r="C89" t="s">
-        <v>198</v>
+        <v>202</v>
       </c>
       <c r="D89" t="s">
         <v>14</v>
       </c>
       <c r="E89" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F89">
         <v>0</v>
@@ -4267,15 +4267,15 @@
         <v>0</v>
       </c>
     </row>
-    <row r="90" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A90" t="s">
         <v>172</v>
       </c>
       <c r="B90" t="s">
-        <v>199</v>
+        <v>203</v>
       </c>
       <c r="C90" t="s">
-        <v>200</v>
+        <v>204</v>
       </c>
       <c r="D90" t="s">
         <v>14</v>
@@ -4296,7 +4296,7 @@
         <v>0</v>
       </c>
       <c r="J90">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K90">
         <v>0</v>
@@ -4307,10 +4307,10 @@
         <v>172</v>
       </c>
       <c r="B91" t="s">
-        <v>201</v>
+        <v>205</v>
       </c>
       <c r="C91" t="s">
-        <v>202</v>
+        <v>206</v>
       </c>
       <c r="D91" t="s">
         <v>14</v>
@@ -4322,19 +4322,19 @@
         <v>0</v>
       </c>
       <c r="G91">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H91">
         <v>0</v>
       </c>
       <c r="I91">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J91">
         <v>1</v>
       </c>
       <c r="K91">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="92" spans="1:11" x14ac:dyDescent="0.3">
@@ -4342,31 +4342,31 @@
         <v>172</v>
       </c>
       <c r="B92" t="s">
-        <v>203</v>
+        <v>207</v>
       </c>
       <c r="C92" t="s">
-        <v>204</v>
+        <v>208</v>
       </c>
       <c r="D92" t="s">
         <v>14</v>
       </c>
       <c r="E92" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F92">
         <v>1</v>
       </c>
       <c r="G92">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H92">
         <v>0</v>
       </c>
       <c r="I92">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J92">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K92">
         <v>0</v>
@@ -4412,28 +4412,28 @@
         <v>172</v>
       </c>
       <c r="B94" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="C94" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="D94" t="s">
         <v>14</v>
       </c>
       <c r="E94" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F94">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G94">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H94">
         <v>0</v>
       </c>
       <c r="I94">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J94">
         <v>1</v>
@@ -4447,34 +4447,34 @@
         <v>172</v>
       </c>
       <c r="B95" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="C95" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="D95" t="s">
         <v>14</v>
       </c>
       <c r="E95" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F95">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G95">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H95">
         <v>0</v>
       </c>
       <c r="I95">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J95">
         <v>1</v>
       </c>
       <c r="K95">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="96" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
@@ -4972,10 +4972,10 @@
         <v>172</v>
       </c>
       <c r="B110" t="s">
-        <v>239</v>
+        <v>235</v>
       </c>
       <c r="C110" t="s">
-        <v>240</v>
+        <v>236</v>
       </c>
       <c r="D110" t="s">
         <v>14</v>
@@ -4990,16 +4990,16 @@
         <v>0</v>
       </c>
       <c r="H110">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I110">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J110">
         <v>1</v>
       </c>
       <c r="K110">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="111" spans="1:11" x14ac:dyDescent="0.3">
@@ -5007,34 +5007,34 @@
         <v>172</v>
       </c>
       <c r="B111" t="s">
-        <v>241</v>
+        <v>237</v>
       </c>
       <c r="C111" t="s">
-        <v>242</v>
+        <v>238</v>
       </c>
       <c r="D111" t="s">
         <v>14</v>
       </c>
       <c r="E111" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F111">
         <v>1</v>
       </c>
       <c r="G111">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H111">
         <v>0</v>
       </c>
       <c r="I111">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J111">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K111">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="112" spans="1:11" x14ac:dyDescent="0.3">
@@ -5042,10 +5042,10 @@
         <v>172</v>
       </c>
       <c r="B112" t="s">
-        <v>243</v>
+        <v>239</v>
       </c>
       <c r="C112" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="D112" t="s">
         <v>14</v>
@@ -5057,10 +5057,10 @@
         <v>0</v>
       </c>
       <c r="G112">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H112">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I112">
         <v>0</v>
@@ -5072,15 +5072,15 @@
         <v>0</v>
       </c>
     </row>
-    <row r="113" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
       <c r="A113" t="s">
         <v>172</v>
       </c>
       <c r="B113" t="s">
-        <v>235</v>
+        <v>241</v>
       </c>
       <c r="C113" t="s">
-        <v>236</v>
+        <v>242</v>
       </c>
       <c r="D113" t="s">
         <v>14</v>
@@ -5089,22 +5089,22 @@
         <v>15</v>
       </c>
       <c r="F113">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G113">
         <v>0</v>
       </c>
       <c r="H113">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I113">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J113">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K113">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="114" spans="1:11" x14ac:dyDescent="0.3">
@@ -5112,10 +5112,10 @@
         <v>172</v>
       </c>
       <c r="B114" t="s">
-        <v>247</v>
+        <v>243</v>
       </c>
       <c r="C114" t="s">
-        <v>248</v>
+        <v>244</v>
       </c>
       <c r="D114" t="s">
         <v>14</v>
@@ -5124,16 +5124,16 @@
         <v>15</v>
       </c>
       <c r="F114">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G114">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H114">
         <v>1</v>
       </c>
       <c r="I114">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J114">
         <v>1</v>
@@ -5147,10 +5147,10 @@
         <v>172</v>
       </c>
       <c r="B115" t="s">
-        <v>249</v>
+        <v>245</v>
       </c>
       <c r="C115" t="s">
-        <v>250</v>
+        <v>246</v>
       </c>
       <c r="D115" t="s">
         <v>14</v>
@@ -5162,7 +5162,7 @@
         <v>0</v>
       </c>
       <c r="G115">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H115">
         <v>0</v>
@@ -5174,7 +5174,7 @@
         <v>1</v>
       </c>
       <c r="K115">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="116" spans="1:11" x14ac:dyDescent="0.3">
@@ -5182,25 +5182,25 @@
         <v>172</v>
       </c>
       <c r="B116" t="s">
-        <v>237</v>
+        <v>247</v>
       </c>
       <c r="C116" t="s">
-        <v>238</v>
+        <v>248</v>
       </c>
       <c r="D116" t="s">
         <v>14</v>
       </c>
       <c r="E116" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F116">
         <v>1</v>
       </c>
       <c r="G116">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H116">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I116">
         <v>1</v>
@@ -5209,7 +5209,7 @@
         <v>1</v>
       </c>
       <c r="K116">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="117" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
@@ -5252,10 +5252,10 @@
         <v>172</v>
       </c>
       <c r="B118" t="s">
-        <v>245</v>
+        <v>249</v>
       </c>
       <c r="C118" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
       <c r="D118" t="s">
         <v>14</v>
@@ -5267,7 +5267,7 @@
         <v>0</v>
       </c>
       <c r="G118">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H118">
         <v>0</v>
@@ -5279,7 +5279,7 @@
         <v>1</v>
       </c>
       <c r="K118">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -5289,7 +5289,12 @@
         <filter val="Vogels"/>
       </filters>
     </filterColumn>
-    <sortState ref="A4:K118">
+    <filterColumn colId="9">
+      <filters>
+        <filter val="1"/>
+      </filters>
+    </filterColumn>
+    <sortState ref="A11:K118">
       <sortCondition ref="B1:B118"/>
     </sortState>
   </autoFilter>

</xml_diff>